<commit_message>
Update Meesho template updated
</commit_message>
<xml_diff>
--- a/main/marketplaces/mysmme/saree-product-import-template.xlsx
+++ b/main/marketplaces/mysmme/saree-product-import-template.xlsx
@@ -10,7 +10,7 @@
   </sheets>
   <definedNames>
     <definedName name="GSTList">'System-Data'!$E$2</definedName>
-    <definedName name="ATTR_BLOUSE">'System-Data'!$G$2:$G$8</definedName>
+    <definedName name="ATTR_BLOUSE">'System-Data'!$G$2:$G$9</definedName>
     <definedName name="ATTR_BLOUSEFABRIC">'System-Data'!$H$2</definedName>
     <definedName name="ATTR_BLOUSEPATTERN">'System-Data'!$I$2:$I$11</definedName>
     <definedName name="ATTR_BORDER">'System-Data'!$J$2:$J$10</definedName>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="467">
   <si>
     <t>VERSION-1.0</t>
   </si>
@@ -318,289 +318,292 @@
     <t>AW-26</t>
   </si>
   <si>
+    <t>Running Blouse</t>
+  </si>
+  <si>
+    <t>Zamato</t>
+  </si>
+  <si>
+    <t>Embellished</t>
+  </si>
+  <si>
+    <t>Big Border</t>
+  </si>
+  <si>
+    <t>100% Acrylic</t>
+  </si>
+  <si>
+    <t>Handloom</t>
+  </si>
+  <si>
+    <t>Bridal</t>
+  </si>
+  <si>
+    <t>Aari Work</t>
+  </si>
+  <si>
+    <t>Checked</t>
+  </si>
+  <si>
+    <t>Abstract</t>
+  </si>
+  <si>
+    <t>Acrylic</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Assam Silk</t>
+  </si>
+  <si>
+    <t>KURTICO</t>
+  </si>
+  <si>
+    <t>Bandhani Saree</t>
+  </si>
+  <si>
+    <t>Beige</t>
+  </si>
+  <si>
+    <t>AW-27</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>Saree with Multiple Blouse</t>
   </si>
   <si>
-    <t>Zamato</t>
-  </si>
-  <si>
-    <t>Embellished</t>
-  </si>
-  <si>
-    <t>Big Border</t>
-  </si>
-  <si>
-    <t>100% Acrylic</t>
-  </si>
-  <si>
-    <t>Handloom</t>
-  </si>
-  <si>
-    <t>Bridal</t>
-  </si>
-  <si>
-    <t>Aari Work</t>
-  </si>
-  <si>
-    <t>Checked</t>
-  </si>
-  <si>
-    <t>Abstract</t>
-  </si>
-  <si>
-    <t>Acrylic</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Assam Silk</t>
-  </si>
-  <si>
-    <t>KURTICO</t>
-  </si>
-  <si>
-    <t>Bandhani Saree</t>
-  </si>
-  <si>
-    <t>Beige</t>
-  </si>
-  <si>
-    <t>AW-27</t>
-  </si>
-  <si>
-    <t/>
+    <t>Embroidered</t>
+  </si>
+  <si>
+    <t>Medium Border</t>
+  </si>
+  <si>
+    <t>100% Cotton</t>
+  </si>
+  <si>
+    <t>Powerloom</t>
+  </si>
+  <si>
+    <t>Casual</t>
+  </si>
+  <si>
+    <t>Applique</t>
+  </si>
+  <si>
+    <t>Colorblocked</t>
+  </si>
+  <si>
+    <t>Ajrakh</t>
+  </si>
+  <si>
+    <t>Art Silk</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Baluchari</t>
+  </si>
+  <si>
+    <t>SHRIJAMYAHAM</t>
+  </si>
+  <si>
+    <t>Bhagalpuri Silk Saree</t>
+  </si>
+  <si>
+    <t>Black</t>
+  </si>
+  <si>
+    <t>AW-28</t>
   </si>
   <si>
     <t>Semi-Stitched Blouse</t>
   </si>
   <si>
-    <t>Embroidered</t>
-  </si>
-  <si>
-    <t>Medium Border</t>
-  </si>
-  <si>
-    <t>100% Cotton</t>
-  </si>
-  <si>
-    <t>Powerloom</t>
-  </si>
-  <si>
-    <t>Casual</t>
-  </si>
-  <si>
-    <t>Applique</t>
-  </si>
-  <si>
-    <t>Colorblocked</t>
-  </si>
-  <si>
-    <t>Ajrakh</t>
-  </si>
-  <si>
-    <t>Art Silk</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>Baluchari</t>
-  </si>
-  <si>
-    <t>SHRIJAMYAHAM</t>
-  </si>
-  <si>
-    <t>Bhagalpuri Silk Saree</t>
-  </si>
-  <si>
-    <t>Black</t>
-  </si>
-  <si>
-    <t>AW-28</t>
+    <t>Jacquard</t>
+  </si>
+  <si>
+    <t>Lace</t>
+  </si>
+  <si>
+    <t>No Border</t>
+  </si>
+  <si>
+    <t>100% Linen</t>
+  </si>
+  <si>
+    <t>Celebrity Inspired</t>
+  </si>
+  <si>
+    <t>Beads &amp; Stones</t>
+  </si>
+  <si>
+    <t>Half &amp; Half</t>
+  </si>
+  <si>
+    <t>Printed</t>
+  </si>
+  <si>
+    <t>Animal</t>
+  </si>
+  <si>
+    <t>Aura Silk</t>
+  </si>
+  <si>
+    <t>Banarasi</t>
+  </si>
+  <si>
+    <t>Saznara</t>
+  </si>
+  <si>
+    <t>Bomkai Saree</t>
+  </si>
+  <si>
+    <t>Blue</t>
+  </si>
+  <si>
+    <t>SS-26</t>
   </si>
   <si>
     <t>Separate Blouse Piece</t>
   </si>
   <si>
-    <t>Jacquard</t>
-  </si>
-  <si>
-    <t>Lace</t>
-  </si>
-  <si>
-    <t>No Border</t>
-  </si>
-  <si>
-    <t>100% Linen</t>
-  </si>
-  <si>
-    <t>Celebrity Inspired</t>
-  </si>
-  <si>
-    <t>Beads &amp; Stones</t>
-  </si>
-  <si>
-    <t>Half &amp; Half</t>
-  </si>
-  <si>
-    <t>Printed</t>
-  </si>
-  <si>
-    <t>Animal</t>
-  </si>
-  <si>
-    <t>Aura Silk</t>
-  </si>
-  <si>
-    <t>Banarasi</t>
-  </si>
-  <si>
-    <t>Saznara</t>
-  </si>
-  <si>
-    <t>Bomkai Saree</t>
-  </si>
-  <si>
-    <t>Blue</t>
-  </si>
-  <si>
-    <t>SS-26</t>
+    <t>Small Border</t>
+  </si>
+  <si>
+    <t>100% Nylon</t>
+  </si>
+  <si>
+    <t>Daily Wear</t>
+  </si>
+  <si>
+    <t>Brocade</t>
+  </si>
+  <si>
+    <t>Self-Design</t>
+  </si>
+  <si>
+    <t>Aztec</t>
+  </si>
+  <si>
+    <t>Balaton Silk</t>
+  </si>
+  <si>
+    <t>Bandhani</t>
+  </si>
+  <si>
+    <t>Bridal Saree</t>
+  </si>
+  <si>
+    <t>Bronze</t>
+  </si>
+  <si>
+    <t>SS-27</t>
   </si>
   <si>
     <t>Stitched Blouse</t>
   </si>
   <si>
-    <t>Small Border</t>
-  </si>
-  <si>
-    <t>100% Nylon</t>
-  </si>
-  <si>
-    <t>Daily Wear</t>
-  </si>
-  <si>
-    <t>Brocade</t>
-  </si>
-  <si>
-    <t>Self-Design</t>
-  </si>
-  <si>
-    <t>Aztec</t>
-  </si>
-  <si>
-    <t>Balaton Silk</t>
-  </si>
-  <si>
-    <t>Bandhani</t>
-  </si>
-  <si>
-    <t>Bridal Saree</t>
-  </si>
-  <si>
-    <t>Bronze</t>
-  </si>
-  <si>
-    <t>SS-27</t>
+    <t>Same as Border</t>
+  </si>
+  <si>
+    <t>100% Polyamide</t>
+  </si>
+  <si>
+    <t>Farewell</t>
+  </si>
+  <si>
+    <t>Brooch</t>
+  </si>
+  <si>
+    <t>Solid</t>
+  </si>
+  <si>
+    <t>Bagh</t>
+  </si>
+  <si>
+    <t>Bamboo</t>
+  </si>
+  <si>
+    <t>Begumpuri</t>
+  </si>
+  <si>
+    <t>Chanderi Saree</t>
+  </si>
+  <si>
+    <t>Brown</t>
+  </si>
+  <si>
+    <t>SS-28</t>
   </si>
   <si>
     <t>Unstitched</t>
   </si>
   <si>
-    <t>Same as Border</t>
-  </si>
-  <si>
-    <t>100% Polyamide</t>
-  </si>
-  <si>
-    <t>Farewell</t>
-  </si>
-  <si>
-    <t>Brooch</t>
-  </si>
-  <si>
-    <t>Solid</t>
-  </si>
-  <si>
-    <t>Bagh</t>
-  </si>
-  <si>
-    <t>Bamboo</t>
-  </si>
-  <si>
-    <t>Begumpuri</t>
-  </si>
-  <si>
-    <t>Chanderi Saree</t>
-  </si>
-  <si>
-    <t>Brown</t>
-  </si>
-  <si>
-    <t>SS-28</t>
+    <t>Same as Pallu</t>
+  </si>
+  <si>
+    <t>100% Polyester</t>
+  </si>
+  <si>
+    <t>Festival</t>
+  </si>
+  <si>
+    <t>Chikankari</t>
+  </si>
+  <si>
+    <t>Striped</t>
+  </si>
+  <si>
+    <t>Bagru Print</t>
+  </si>
+  <si>
+    <t>Banarasi Silk</t>
+  </si>
+  <si>
+    <t>Belt Saree</t>
+  </si>
+  <si>
+    <t>Chiffon Saree</t>
+  </si>
+  <si>
+    <t>Burgundy</t>
   </si>
   <si>
     <t>Without Blouse</t>
   </si>
   <si>
-    <t>Same as Pallu</t>
-  </si>
-  <si>
-    <t>100% Polyester</t>
-  </si>
-  <si>
-    <t>Festival</t>
-  </si>
-  <si>
-    <t>Chikankari</t>
-  </si>
-  <si>
-    <t>Striped</t>
-  </si>
-  <si>
-    <t>Bagru Print</t>
-  </si>
-  <si>
-    <t>Banarasi Silk</t>
-  </si>
-  <si>
-    <t>Belt Saree</t>
-  </si>
-  <si>
-    <t>Chiffon Saree</t>
-  </si>
-  <si>
-    <t>Burgundy</t>
+    <t>Same as Saree</t>
+  </si>
+  <si>
+    <t>Temple Border</t>
+  </si>
+  <si>
+    <t>100% Rayon</t>
+  </si>
+  <si>
+    <t>Office Wear</t>
+  </si>
+  <si>
+    <t>Cutwork</t>
+  </si>
+  <si>
+    <t>Bangalori Silk</t>
+  </si>
+  <si>
+    <t>Bishnupuri</t>
+  </si>
+  <si>
+    <t>Chikankari Saree</t>
+  </si>
+  <si>
+    <t>Camel Brown</t>
   </si>
   <si>
     <t>Without Blouse abc</t>
-  </si>
-  <si>
-    <t>Same as Saree</t>
-  </si>
-  <si>
-    <t>Temple Border</t>
-  </si>
-  <si>
-    <t>100% Rayon</t>
-  </si>
-  <si>
-    <t>Office Wear</t>
-  </si>
-  <si>
-    <t>Cutwork</t>
-  </si>
-  <si>
-    <t>Bangalori Silk</t>
-  </si>
-  <si>
-    <t>Bishnupuri</t>
-  </si>
-  <si>
-    <t>Chikankari Saree</t>
-  </si>
-  <si>
-    <t>Camel Brown</t>
   </si>
   <si>
     <t>Woven Design</t>
@@ -3966,32 +3969,35 @@
       <c r="E9" t="s">
         <v>112</v>
       </c>
+      <c r="G9" t="s">
+        <v>190</v>
+      </c>
       <c r="I9" t="s">
         <v>162</v>
       </c>
       <c r="J9" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="L9" t="s">
+        <v>192</v>
+      </c>
+      <c r="N9" t="s">
+        <v>193</v>
+      </c>
+      <c r="O9" t="s">
+        <v>194</v>
+      </c>
+      <c r="P9" t="s">
         <v>191</v>
       </c>
-      <c r="N9" t="s">
-        <v>192</v>
-      </c>
-      <c r="O9" t="s">
-        <v>193</v>
-      </c>
-      <c r="P9" t="s">
-        <v>190</v>
-      </c>
       <c r="R9" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="S9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="U9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
@@ -3999,10 +4005,10 @@
         <v>112</v>
       </c>
       <c r="B10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D10" t="s">
         <v>112</v>
@@ -4011,31 +4017,31 @@
         <v>112</v>
       </c>
       <c r="I10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J10" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="L10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="N10" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="O10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="P10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="R10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="S10" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="U10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
@@ -4043,10 +4049,10 @@
         <v>112</v>
       </c>
       <c r="B11" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C11" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D11" t="s">
         <v>112</v>
@@ -4055,25 +4061,25 @@
         <v>112</v>
       </c>
       <c r="I11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L11" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="N11" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="O11" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="R11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="S11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="U11" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
@@ -4081,10 +4087,10 @@
         <v>112</v>
       </c>
       <c r="B12" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C12" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D12" t="s">
         <v>112</v>
@@ -4093,22 +4099,22 @@
         <v>112</v>
       </c>
       <c r="L12" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="N12" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="O12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="R12" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="S12" t="s">
         <v>149</v>
       </c>
       <c r="U12" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
@@ -4116,10 +4122,10 @@
         <v>112</v>
       </c>
       <c r="B13" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C13" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D13" t="s">
         <v>112</v>
@@ -4128,19 +4134,19 @@
         <v>112</v>
       </c>
       <c r="L13" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="O13" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="R13" t="s">
         <v>103</v>
       </c>
       <c r="S13" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="U13" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
@@ -4148,10 +4154,10 @@
         <v>112</v>
       </c>
       <c r="B14" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C14" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D14" t="s">
         <v>112</v>
@@ -4160,19 +4166,19 @@
         <v>112</v>
       </c>
       <c r="L14" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="O14" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="R14" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="S14" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="U14" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
@@ -4180,10 +4186,10 @@
         <v>112</v>
       </c>
       <c r="B15" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C15" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D15" t="s">
         <v>112</v>
@@ -4192,19 +4198,19 @@
         <v>112</v>
       </c>
       <c r="L15" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="O15" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="R15" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="S15" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="U15" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
@@ -4212,10 +4218,10 @@
         <v>112</v>
       </c>
       <c r="B16" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C16" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D16" t="s">
         <v>112</v>
@@ -4224,19 +4230,19 @@
         <v>112</v>
       </c>
       <c r="L16" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="O16" t="s">
         <v>131</v>
       </c>
       <c r="R16" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="S16" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="U16" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
@@ -4244,10 +4250,10 @@
         <v>112</v>
       </c>
       <c r="B17" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C17" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D17" t="s">
         <v>112</v>
@@ -4256,19 +4262,19 @@
         <v>112</v>
       </c>
       <c r="L17" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="O17" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="R17" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="S17" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="U17" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
@@ -4276,10 +4282,10 @@
         <v>112</v>
       </c>
       <c r="B18" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C18" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D18" t="s">
         <v>112</v>
@@ -4288,19 +4294,19 @@
         <v>112</v>
       </c>
       <c r="L18" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="O18" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="R18" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="S18" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="U18" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
@@ -4308,10 +4314,10 @@
         <v>112</v>
       </c>
       <c r="B19" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C19" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D19" t="s">
         <v>112</v>
@@ -4320,19 +4326,19 @@
         <v>112</v>
       </c>
       <c r="L19" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="O19" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="R19" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="S19" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="U19" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
@@ -4340,10 +4346,10 @@
         <v>112</v>
       </c>
       <c r="B20" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C20" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D20" t="s">
         <v>112</v>
@@ -4352,19 +4358,19 @@
         <v>112</v>
       </c>
       <c r="L20" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="O20" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="R20" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="S20" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="U20" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
@@ -4372,10 +4378,10 @@
         <v>112</v>
       </c>
       <c r="B21" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C21" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D21" t="s">
         <v>112</v>
@@ -4384,19 +4390,19 @@
         <v>112</v>
       </c>
       <c r="L21" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="O21" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="R21" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="S21" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="U21" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
@@ -4404,10 +4410,10 @@
         <v>112</v>
       </c>
       <c r="B22" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C22" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D22" t="s">
         <v>112</v>
@@ -4416,16 +4422,16 @@
         <v>112</v>
       </c>
       <c r="O22" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="R22" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="S22" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="U22" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
@@ -4433,10 +4439,10 @@
         <v>112</v>
       </c>
       <c r="B23" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C23" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D23" t="s">
         <v>112</v>
@@ -4445,16 +4451,16 @@
         <v>112</v>
       </c>
       <c r="O23" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="R23" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="S23" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="U23" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
@@ -4462,10 +4468,10 @@
         <v>112</v>
       </c>
       <c r="B24" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C24" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D24" t="s">
         <v>112</v>
@@ -4474,16 +4480,16 @@
         <v>112</v>
       </c>
       <c r="O24" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="R24" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="S24" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="U24" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
@@ -4491,10 +4497,10 @@
         <v>112</v>
       </c>
       <c r="B25" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C25" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D25" t="s">
         <v>112</v>
@@ -4503,16 +4509,16 @@
         <v>112</v>
       </c>
       <c r="O25" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="R25" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="S25" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="U25" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
@@ -4520,10 +4526,10 @@
         <v>112</v>
       </c>
       <c r="B26" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C26" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D26" t="s">
         <v>112</v>
@@ -4532,16 +4538,16 @@
         <v>112</v>
       </c>
       <c r="O26" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="R26" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="S26" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="U26" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
@@ -4549,10 +4555,10 @@
         <v>112</v>
       </c>
       <c r="B27" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C27" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D27" t="s">
         <v>112</v>
@@ -4561,16 +4567,16 @@
         <v>112</v>
       </c>
       <c r="O27" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="R27" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="S27" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="U27" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
@@ -4578,10 +4584,10 @@
         <v>112</v>
       </c>
       <c r="B28" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C28" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D28" t="s">
         <v>112</v>
@@ -4590,16 +4596,16 @@
         <v>112</v>
       </c>
       <c r="O28" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="R28" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="S28" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="U28" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -4607,10 +4613,10 @@
         <v>112</v>
       </c>
       <c r="B29" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C29" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D29" t="s">
         <v>112</v>
@@ -4619,16 +4625,16 @@
         <v>112</v>
       </c>
       <c r="O29" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="R29" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="S29" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="U29" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
@@ -4636,10 +4642,10 @@
         <v>112</v>
       </c>
       <c r="B30" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C30" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D30" t="s">
         <v>112</v>
@@ -4648,16 +4654,16 @@
         <v>112</v>
       </c>
       <c r="O30" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="R30" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="S30" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="U30" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
@@ -4665,10 +4671,10 @@
         <v>112</v>
       </c>
       <c r="B31" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C31" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D31" t="s">
         <v>112</v>
@@ -4677,13 +4683,13 @@
         <v>112</v>
       </c>
       <c r="R31" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="S31" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="U31" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
@@ -4691,10 +4697,10 @@
         <v>112</v>
       </c>
       <c r="B32" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C32" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D32" t="s">
         <v>112</v>
@@ -4703,13 +4709,13 @@
         <v>112</v>
       </c>
       <c r="R32" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="S32" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="U32" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
@@ -4717,10 +4723,10 @@
         <v>112</v>
       </c>
       <c r="B33" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C33" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D33" t="s">
         <v>112</v>
@@ -4729,13 +4735,13 @@
         <v>112</v>
       </c>
       <c r="R33" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="S33" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="U33" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
@@ -4743,10 +4749,10 @@
         <v>112</v>
       </c>
       <c r="B34" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C34" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D34" t="s">
         <v>112</v>
@@ -4755,13 +4761,13 @@
         <v>112</v>
       </c>
       <c r="R34" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="S34" t="s">
         <v>130</v>
       </c>
       <c r="U34" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
@@ -4772,7 +4778,7 @@
         <v>112</v>
       </c>
       <c r="C35" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D35" t="s">
         <v>112</v>
@@ -4781,13 +4787,13 @@
         <v>112</v>
       </c>
       <c r="R35" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="S35" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="U35" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
@@ -4798,7 +4804,7 @@
         <v>112</v>
       </c>
       <c r="C36" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D36" t="s">
         <v>112</v>
@@ -4807,13 +4813,13 @@
         <v>112</v>
       </c>
       <c r="R36" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="S36" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="U36" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
@@ -4824,7 +4830,7 @@
         <v>112</v>
       </c>
       <c r="C37" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D37" t="s">
         <v>112</v>
@@ -4833,13 +4839,13 @@
         <v>112</v>
       </c>
       <c r="R37" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="S37" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="U37" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
@@ -4850,7 +4856,7 @@
         <v>112</v>
       </c>
       <c r="C38" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D38" t="s">
         <v>112</v>
@@ -4862,10 +4868,10 @@
         <v>162</v>
       </c>
       <c r="S38" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="U38" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
@@ -4876,7 +4882,7 @@
         <v>112</v>
       </c>
       <c r="C39" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D39" t="s">
         <v>112</v>
@@ -4885,13 +4891,13 @@
         <v>112</v>
       </c>
       <c r="R39" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="S39" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="U39" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
@@ -4902,7 +4908,7 @@
         <v>112</v>
       </c>
       <c r="C40" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D40" t="s">
         <v>112</v>
@@ -4911,13 +4917,13 @@
         <v>112</v>
       </c>
       <c r="R40" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="S40" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="U40" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
@@ -4928,7 +4934,7 @@
         <v>112</v>
       </c>
       <c r="C41" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D41" t="s">
         <v>112</v>
@@ -4937,13 +4943,13 @@
         <v>112</v>
       </c>
       <c r="R41" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="S41" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="U41" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
@@ -4954,7 +4960,7 @@
         <v>112</v>
       </c>
       <c r="C42" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D42" t="s">
         <v>112</v>
@@ -4963,13 +4969,13 @@
         <v>112</v>
       </c>
       <c r="R42" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="S42" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="U42" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
@@ -4980,7 +4986,7 @@
         <v>112</v>
       </c>
       <c r="C43" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="D43" t="s">
         <v>112</v>
@@ -4989,13 +4995,13 @@
         <v>112</v>
       </c>
       <c r="R43" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="S43" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="U43" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
@@ -5006,7 +5012,7 @@
         <v>112</v>
       </c>
       <c r="C44" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D44" t="s">
         <v>112</v>
@@ -5015,10 +5021,10 @@
         <v>112</v>
       </c>
       <c r="S44" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="U44" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
@@ -5029,7 +5035,7 @@
         <v>112</v>
       </c>
       <c r="C45" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D45" t="s">
         <v>112</v>
@@ -5038,10 +5044,10 @@
         <v>112</v>
       </c>
       <c r="S45" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="U45" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
@@ -5052,7 +5058,7 @@
         <v>112</v>
       </c>
       <c r="C46" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="D46" t="s">
         <v>112</v>
@@ -5061,10 +5067,10 @@
         <v>112</v>
       </c>
       <c r="S46" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="U46" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
@@ -5075,7 +5081,7 @@
         <v>112</v>
       </c>
       <c r="C47" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="D47" t="s">
         <v>112</v>
@@ -5084,10 +5090,10 @@
         <v>112</v>
       </c>
       <c r="S47" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="U47" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
@@ -5098,7 +5104,7 @@
         <v>112</v>
       </c>
       <c r="C48" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D48" t="s">
         <v>112</v>
@@ -5110,7 +5116,7 @@
         <v>131</v>
       </c>
       <c r="U48" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
@@ -5121,7 +5127,7 @@
         <v>112</v>
       </c>
       <c r="C49" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="D49" t="s">
         <v>112</v>
@@ -5130,10 +5136,10 @@
         <v>112</v>
       </c>
       <c r="S49" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="U49" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
@@ -5144,7 +5150,7 @@
         <v>112</v>
       </c>
       <c r="C50" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D50" t="s">
         <v>112</v>
@@ -5153,10 +5159,10 @@
         <v>112</v>
       </c>
       <c r="S50" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="U50" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -5167,7 +5173,7 @@
         <v>112</v>
       </c>
       <c r="C51" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D51" t="s">
         <v>112</v>
@@ -5176,294 +5182,294 @@
         <v>112</v>
       </c>
       <c r="S51" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="U51" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="52" spans="19:21" x14ac:dyDescent="0.25">
       <c r="S52" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="U52" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="53" spans="19:21" x14ac:dyDescent="0.25">
       <c r="S53" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="U53" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="54" spans="19:21" x14ac:dyDescent="0.25">
       <c r="S54" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="U54" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="55" spans="19:21" x14ac:dyDescent="0.25">
       <c r="S55" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="U55" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
     </row>
     <row r="56" spans="19:21" x14ac:dyDescent="0.25">
       <c r="S56" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="U56" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="57" spans="19:21" x14ac:dyDescent="0.25">
       <c r="S57" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="U57" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="58" spans="19:21" x14ac:dyDescent="0.25">
       <c r="S58" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="U58" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="59" spans="19:21" x14ac:dyDescent="0.25">
       <c r="S59" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="U59" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="60" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S60" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="61" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S61" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="62" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S62" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="63" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S63" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
     <row r="64" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S64" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="65" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S65" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="66" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S66" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
     </row>
     <row r="67" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S67" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="68" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S68" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
     </row>
     <row r="69" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S69" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="70" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S70" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="71" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S71" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="72" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S72" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="73" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S73" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="74" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S74" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="75" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S75" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="76" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S76" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="77" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S77" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="78" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S78" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="79" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S79" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="80" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S80" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="81" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S81" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="82" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S82" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="83" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S83" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="84" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S84" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="85" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S85" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="86" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S86" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="87" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S87" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="88" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S88" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="89" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S89" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="90" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S90" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="91" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S91" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
     <row r="92" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S92" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
     <row r="93" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S93" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="94" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S94" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
     </row>
     <row r="95" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S95" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
     </row>
     <row r="96" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S96" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="97" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S97" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="98" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S98" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
     </row>
     <row r="99" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S99" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="100" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S100" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="101" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S101" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
     </row>
     <row r="102" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S102" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
     </row>
     <row r="103" spans="19:19" x14ac:dyDescent="0.25">
       <c r="S103" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="104" spans="19:19" x14ac:dyDescent="0.25">

</xml_diff>